<commit_message>
BOMs: threaded spacers under review (linked ones measure ~5.05 mm); sanding note for anyone who has them
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CF Version/SV08_CF6_BOM_from_STEP.xlsx
+++ b/CF Version/SV08_CF6_BOM_from_STEP.xlsx
@@ -943,7 +943,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint.</t>
+          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. UNDER REVIEW: the linked spacers measure about 5.05 mm across (anodised aluminium), too big for the 4.992-5.000 mm bore of a 695 bearing, so they won't slide in. We're evaluating replacements. If you already have them, sand the last ~2 mm of each end (the only part that goes into the bearings) down to about 4.990-4.995 mm: spin it in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go, and stop when it presses into a bearing with firm thumb pressure. Don't force an oversize spacer in; that loads the bearing balls.</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head.</t>
+          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. UNDER REVIEW: the linked spacers measure about 5.05 mm across (anodised aluminium), too big for the 4.992-5.000 mm bore of a 695 bearing, so they won't slide in. We're evaluating replacements. If you already have them, sand the last ~2 mm of each end (the only part that goes into the bearings) down to about 4.990-4.995 mm: spin it in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go, and stop when it presses into a bearing with firm thumb pressure. Don't force an oversize spacer in; that loads the bearing balls.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BOMs: 5 mm slip-fit dowel (40 mm XY, 30 mm front) as an alternative to the threaded spacers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CF Version/SV08_CF6_BOM_from_STEP.xlsx
+++ b/CF Version/SV08_CF6_BOM_from_STEP.xlsx
@@ -943,7 +943,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. UNDER REVIEW: the linked spacers measure about 5.05 mm across (anodised aluminium), too big for the 4.992-5.000 mm bore of a 695 bearing, so they won't slide in. We're evaluating replacements. If you already have them, sand the last ~2 mm of each end (the only part that goes into the bearings) down to about 4.990-4.995 mm: spin it in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go, and stop when it presses into a bearing with firm thumb pressure. Don't force an oversize spacer in; that loads the bearing balls.</t>
+          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. UNDER REVIEW: the linked spacers measure about 5.05 mm across (anodised aluminium), too big for the 4.992-5.000 mm bore of a 695 bearing, so they won't slide in. We're evaluating replacements. If you already have them, sand the last ~2 mm of each end (the only part that goes into the bearings) down to about 4.990-4.995 mm: spin it in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go, and stop when it presses into a bearing with firm thumb pressure. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 40 mm long, works in place of the spacer and its two flat-head screws. At 40 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. UNDER REVIEW: the linked spacers measure about 5.05 mm across (anodised aluminium), too big for the 4.992-5.000 mm bore of a 695 bearing, so they won't slide in. We're evaluating replacements. If you already have them, sand the last ~2 mm of each end (the only part that goes into the bearings) down to about 4.990-4.995 mm: spin it in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go, and stop when it presses into a bearing with firm thumb pressure. Don't force an oversize spacer in; that loads the bearing balls.</t>
+          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. UNDER REVIEW: the linked spacers measure about 5.05 mm across (anodised aluminium), too big for the 4.992-5.000 mm bore of a 695 bearing, so they won't slide in. We're evaluating replacements. If you already have them, sand the last ~2 mm of each end (the only part that goes into the bearings) down to about 4.990-4.995 mm: spin it in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go, and stop when it presses into a bearing with firm thumb pressure. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 30 mm long, works in place of the spacer and its two flat-head screws. At 30 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BOMs: threaded spacers confirmed working once sanded full length to fit (pulleys must slide over them too)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CF Version/SV08_CF6_BOM_from_STEP.xlsx
+++ b/CF Version/SV08_CF6_BOM_from_STEP.xlsx
@@ -943,7 +943,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. UNDER REVIEW: the linked spacers measure about 5.05 mm across (anodised aluminium), too big for the 4.992-5.000 mm bore of a 695 bearing, so they won't slide in. We're evaluating replacements. If you already have them, sand the last ~2 mm of each end (the only part that goes into the bearings) down to about 4.990-4.995 mm: spin it in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go, and stop when it presses into a bearing with firm thumb pressure. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 40 mm long, works in place of the spacer and its two flat-head screws. At 40 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 40 mm long, works in place of the spacer and its two flat-head screws. At 40 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. UNDER REVIEW: the linked spacers measure about 5.05 mm across (anodised aluminium), too big for the 4.992-5.000 mm bore of a 695 bearing, so they won't slide in. We're evaluating replacements. If you already have them, sand the last ~2 mm of each end (the only part that goes into the bearings) down to about 4.990-4.995 mm: spin it in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go, and stop when it presses into a bearing with firm thumb pressure. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 30 mm long, works in place of the spacer and its two flat-head screws. At 30 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 30 mm long, works in place of the spacer and its two flat-head screws. At 30 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BOMs: stock extrusion compatibility notes; stock 345 mm gantry X fits with a 6 mm OD spacer at each end
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CF Version/SV08_CF6_BOM_from_STEP.xlsx
+++ b/CF Version/SV08_CF6_BOM_from_STEP.xlsx
@@ -1339,7 +1339,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>6mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.</t>
+          <t>6mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions. Optional: use a 6mm OD (or smaller) spacer for the one nearest each end of the Gantry X extrusion (2 total) and the stock 345mm extrusion fits without cutting.</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,11 @@
         </is>
       </c>
       <c r="D71" s="2" t="n"/>
-      <c r="E71" s="2" t="n"/>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Stock extrusion works: the front and back motor-mount bolt holes line up with its existing holes.</t>
+        </is>
+      </c>
     </row>
     <row r="72" s="6">
       <c r="A72" s="2" t="inlineStr">
@@ -1820,7 +1824,7 @@
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts.</t>
+          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts. The back motor-mount bolt holes line up with the stock extrusion's existing holes. To use the stock 345mm extrusion without cutting it, fit a 6mm OD (or smaller) M3 x 20mm spacer in the spot nearest each end of this extrusion (one per back corner) instead of an 8mm one.</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1843,11 @@
         </is>
       </c>
       <c r="D73" s="2" t="n"/>
-      <c r="E73" s="2" t="n"/>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>The XY joints don't line up with the stock extrusion's holes (different bolt pattern). Either mount them with M4 T-nuts in the slots, or replace this extrusion with one drilled to match.</t>
+        </is>
+      </c>
     </row>
     <row r="74" s="6">
       <c r="A74" s="7" t="inlineStr">

</xml_diff>

<commit_message>
CF: Chicago bolt live idler shafts, XY holes match the stock toolhead extrusion, CF printed parts 3MF
CF fronts and XY joints use the M5x30/M5x40 Chicago bolt bases with M4x8 ultra-thin heads
(spans 30/40 exact, 0.4 mm under the front motors); XY M4 holes moved 0.99 mm to 5 / 25 mm
from the stock toolhead extrusion ends (outlines +1.19 mm); XY spacer re-exported. CF BOM:
Live Idler Shafts section and stock toolhead note. Accepted: XY retainer floors 1.00 mm,
shifted XY Left walls, and the front-bottom 0.40 mm retainer floors for a test cut.
New CF Printed Parts.3mf, STL previews, renders, README notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CF Version/SV08_CF6_BOM_from_STEP.xlsx
+++ b/CF Version/SV08_CF6_BOM_from_STEP.xlsx
@@ -653,21 +653,21 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>M3 x 10mm Ultra Thin Flat Head (.8-1mm)</t>
+          <t>M4x8 Ultra Thin Flat Head</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0H61WCTBX</t>
+          <t>https://amazon.com/dp/B0H61X7SWB</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Ultra-thin head (.8-1mm). 2 per front motor assembly and 2 per XY joint. Use threadlocker: blue (medium, removable) recommended; red (high strength) only for a permanent build, since removing it takes heat that can damage bearings and printed parts.</t>
+          <t>Screw end of each Chicago bolt live idler shaft (1 per front motor assembly and 1 per XY joint). 1.2mm head, thin enough to clear the front motors. Use threadlocker: blue (medium, removable) recommended; red (high strength) only for a permanent build, since removing it takes heat that can damage the bearings.</t>
         </is>
       </c>
     </row>
@@ -872,14 +872,14 @@
     <row r="22" s="6">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Fasteners - Threaded Rods</t>
+          <t>Live Idler Shafts</t>
         </is>
       </c>
     </row>
     <row r="23" s="6">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Threaded Rods</t>
+          <t>Live Idler Shafts</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
@@ -887,24 +887,24 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>M3 Internally Threaded Spacer (5mm OD | 35mm Tall)</t>
+          <t>M5x40 Chicago Bolt Base</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0D3HWQ2GF</t>
+          <t>https://amazon.com/dp/B0FLJNY14R</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 40 mm long, works in place of the spacer and its two flat-head screws. At 40 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+          <t>Live idler shaft in the XY joints (1 per joint). 304 stainless Chicago screw: the 5mm x 40mm barrel runs the full width of both bearings, its head on one bearing and an M4x8 Ultra Thin Flat Head on the other, so the bearings are clamped and the idler can't float. Pack of 20. The M4x4 screws in the pack aren't used: their 2mm heads don't clear the front motors, so the ultra-thin heads are used everywhere. ALTERNATIVES (not as good): an M3 internally threaded spacer, 5mm OD x 35mm (amazon.com/dp/B0D3HWQ2GF), clamped by 2x M3 x 10mm ultra-thin flat heads (amazon.com/dp/B0H61WCTBX). The anodised spacers measure about 5.05mm, so sand the whole length in a drill (400-600 grit) until it presses into a bearing with firm thumb pressure and the pulley slides over it. Or a 5mm h6/h7 slip-fit dowel / ground shaft, 40mm long: it fits, but it's held only by the pulley set screws, so the idler can float up and down under belt tension, which causes vibration.</t>
         </is>
       </c>
     </row>
     <row r="24" s="6">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Threaded Rods</t>
+          <t>Live Idler Shafts</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
@@ -912,17 +912,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>M3 Internally Threaded Spacer (5mm OD | 25mm Tall)</t>
+          <t>M5x30 Chicago Bolt Base</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0D3HVVJPN</t>
+          <t>https://amazon.com/dp/B0FLJQP39V</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 30 mm long, works in place of the spacer and its two flat-head screws. At 30 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+          <t>Live idler shaft in the front motor assemblies (1 per side). 304 stainless Chicago screw: the 5mm x 30mm barrel runs the full width of both bearings, head at the bottom and an M4x8 Ultra Thin Flat Head at the top, 0.4mm under the motor. Pack of 20; the M4x4 screws in the pack aren't used (their 2mm heads don't clear the motor). ALTERNATIVES (not as good): an M3 internally threaded spacer, 5mm OD x 25mm (amazon.com/dp/B0D3HVVJPN), clamped by 2x M3 x 10mm ultra-thin flat heads (amazon.com/dp/B0H61WCTBX). The anodised spacers measure about 5.05mm, so sand the whole length in a drill (400-600 grit) until it presses into a bearing with firm thumb pressure and the pulley slides over it. Or a 5mm h6/h7 slip-fit dowel / ground shaft, 30mm long: it fits, but it's held only by the pulley set screws, so the idler can float up and down under belt tension, which causes vibration.</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>The XY joints don't line up with the stock extrusion's holes (different bolt pattern). Either mount them with M4 T-nuts in the slots, or replace this extrusion with one drilled to match.</t>
+          <t>Stock extrusion works: the XY joint bolt holes line up with its existing holes (5mm and 25mm from each end).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CF: M3 hex nuts in hex pockets replace the PEM standoffs
All 12 CF plates: SO-M3-3ZI / SO-M3-6ZI pockets become M3 nut pockets (5.9 mm A/F, R1 corners,
2.5 mm deep, 2.4 mm at the front-bottom retainers for a 1.0 mm floor; 1 mm lead-in chamfer;
3.2 mm through holes). 36 M3 nuts in the assemblies and main; every screw gets full thread
except the lever-arm screws (2.1 of 2.4 mm, accepted). Collisions unchanged.
BOM: PEM section replaced by an M3 Nut row. Accepted list: front walls/floors updated for the
nut pockets. READMEs: nut pockets instead of PEMs, glue note instead of epoxy, CF hole guide
with current bearing-step depths. STL previews and renders regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CF Version/SV08_CF6_BOM_from_STEP.xlsx
+++ b/CF Version/SV08_CF6_BOM_from_STEP.xlsx
@@ -502,7 +502,7 @@
     <row r="2" ht="30" customHeight="1" s="6">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>From the STEP tree. Z Carriages excluded, D2F-L switches counted as one unit each. Carbon fiber version: the 12 gantry plates and 5mm XY spacers are cut from 6mm CF; PEM self-clinching standoffs replace the heat-set inserts. Draft generated from the Printed BOM; review notes and links.</t>
+          <t>From the STEP tree. Z Carriages excluded, D2F-L switches counted as one unit each. Carbon fiber version: the 12 gantry plates and 5mm XY spacers are cut from 6mm CF; standard M3 hex nuts in hex pockets replace the heat-set inserts. Draft generated from the Printed BOM; review notes and links.</t>
         </is>
       </c>
     </row>
@@ -976,66 +976,84 @@
       <c r="E27" s="2" t="n"/>
     </row>
     <row r="28" s="6">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Inserts - Self-Clinching (PEM)</t>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Nuts</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>M3 Nut</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0F9FC4563</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Standard M3 hex nuts (ISO 4032: 5.5mm across flats, up to 2.4mm thick) in hex pockets in the CF plates, in place of the PEM standoffs: bearing retainers, shoulder bolts and lever-arm screws. The pockets are 5.9mm across flats, so a dab of glue holds a nut in place while you assemble.</t>
         </is>
       </c>
     </row>
     <row r="29" s="6">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Self-Clinching</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>SO-M3-3ZI Insert</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/PEM/SO-M3-3ZI</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>PEM self-clinching standoff, pressed into the CF plates. Replaces the heat-set inserts of the printed version.</t>
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Washers &amp; Shims</t>
         </is>
       </c>
     </row>
     <row r="30" s="6">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Self-Clinching</t>
+          <t>Washers &amp; Shims</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>SO-M3-6ZI Insert</t>
+          <t>M5 Washer (5mm ID | 10mm OD | 1mm Tall)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/PEM/SO-M3-6ZI</t>
+          <t>https://amazon.com/dp/B07WZ5WQCG</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>PEM self-clinching standoff, pressed into the CF plates. Replaces the heat-set inserts of the printed version.</t>
+          <t>Includes the 36 bearing-stack shims, now named M5 Washer.</t>
         </is>
       </c>
     </row>
     <row r="31" s="6">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Washers &amp; Shims</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>M4 Washer (4mm ID | 9mm OD | 1mm Tall)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0DK6KXB6W</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>.8mm more common and acceptable swap, OD matters</t>
         </is>
       </c>
     </row>
@@ -1046,23 +1064,19 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>M5 Washer (5mm ID | 10mm OD | 1mm Tall)</t>
+          <t>M3 Washer (3mm ID | 7mm OD | .5-.6mm Tall)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B07WZ5WQCG</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Includes the 36 bearing-stack shims, now named M5 Washer.</t>
-        </is>
-      </c>
+          <t>https://amazon.com/dp/B0C3TJ7PWT</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
     </row>
     <row r="33" s="6">
       <c r="A33" s="2" t="inlineStr">
@@ -1071,225 +1085,229 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>M4 Washer (4mm ID | 9mm OD | 1mm Tall)</t>
+          <t>M3 Shim (3mm ID | 5mm OD | .2mm Tall)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0DK6KXB6W</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>.8mm more common and acceptable swap, OD matters</t>
-        </is>
-      </c>
+          <t>https://amazon.com/dp/B08ZYP1TK4</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n"/>
     </row>
     <row r="34" s="6">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Washers &amp; Shims</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>M3 Washer (3mm ID | 7mm OD | .5-.6mm Tall)</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0C3TJ7PWT</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n"/>
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Bearings</t>
+        </is>
+      </c>
     </row>
     <row r="35" s="6">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Washers &amp; Shims</t>
+          <t>Bearings</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>M3 Shim (3mm ID | 5mm OD | .2mm Tall)</t>
+          <t>695-2RS Flanged Bearing</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B08ZYP1TK4</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="n"/>
+          <t>https://amazon.com/dp/B0CGXF48ZZ</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Includes the 12 loose bearings named F695-2RS Bearing Single in CAD (36 stacked + 12 loose).</t>
+        </is>
+      </c>
     </row>
     <row r="36" s="6">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Bearings</t>
         </is>
       </c>
+      <c r="B36" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>MR63ZZ Bearing 3x6x2.5mm</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0DY11G865</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n"/>
     </row>
     <row r="37" s="6">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Bearings</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>695-2RS Flanged Bearing</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0CGXF48ZZ</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Includes the 12 loose bearings named F695-2RS Bearing Single in CAD (36 stacked + 12 loose).</t>
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Pulleys</t>
         </is>
       </c>
     </row>
     <row r="38" s="6">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Bearings</t>
+          <t>Pulleys</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>MR63ZZ Bearing 3x6x2.5mm</t>
+          <t>GT2 20-Tooth Pulley Set-Screw Version</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0DY11G865</t>
+          <t>https://amazon.com/dp/B0GWLM6FD6</t>
         </is>
       </c>
       <c r="E38" s="2" t="n"/>
     </row>
     <row r="39" s="6">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Pulleys</t>
         </is>
       </c>
+      <c r="B39" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>GT2 20-Tooth Pulley - Live Idler Version</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256803833151466.html</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Make sure you select Bore 5mm Width 6mm. Uses 2x M2 x 2mm Set Screws each (4 total). Pulley body recovered from an unnamed STEP node (one per XY Joint)</t>
+        </is>
+      </c>
     </row>
     <row r="40" s="6">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Pulleys</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>GT2 20-Tooth Pulley Set-Screw Version</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0GWLM6FD6</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="n"/>
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Belts</t>
+        </is>
+      </c>
     </row>
     <row r="41" s="6">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Pulleys</t>
+          <t>Belts</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>GT2 20-Tooth Pulley - Live Idler Version</t>
+          <t>Bottom Belt 2.1m</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.us/item/3256803833151466.html</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>Make sure you select Bore 5mm Width 6mm. Uses 2x M2 x 2mm Set Screws each (4 total). Pulley body recovered from an unnamed STEP node (one per XY Joint)</t>
-        </is>
-      </c>
+          <t>https://amazon.com/dp/B07CDDPCM8</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n"/>
     </row>
     <row r="42" s="6">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Belts</t>
         </is>
       </c>
+      <c r="B42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Top Belt 2.1m</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B07CDDPCM8</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n"/>
     </row>
     <row r="43" s="6">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Belts</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Bottom Belt 2.1m</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B07CDDPCM8</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n"/>
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Spacers (Aluminum)</t>
+        </is>
+      </c>
     </row>
     <row r="44" s="6">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Belts</t>
+          <t>Spacers (Aluminum)</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Top Belt 2.1m</t>
+          <t>M5 Spacer 10mm OD 10mm Tall</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B07CDDPCM8</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n"/>
+          <t>https://www.aliexpress.com/item/3256802878592600.html</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>8mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.. If purchasing from Aliexpress be sure to select 5.1x10x10</t>
+        </is>
+      </c>
     </row>
     <row r="45" s="6">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Spacers (Aluminum)</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>M3 Spacer 8mm OD 20mm Tall</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0F8QLBKYC</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>6mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions. Optional: use a 6mm OD (or smaller) spacer for the one nearest each end of the Gantry X extrusion (2 total) and the stock 345mm extrusion fits without cutting.</t>
         </is>
       </c>
     </row>
@@ -1300,21 +1318,21 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>M5 Spacer 10mm OD 10mm Tall</t>
+          <t>M5 Spacer 8mm OD 20mm Tall</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/3256802878592600.html</t>
+          <t>https://amazon.com/dp/B0CRL77N5C</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>8mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.. If purchasing from Aliexpress be sure to select 5.1x10x10</t>
+          <t>Purchase preferred. Printed as alternative with same dimensions.</t>
         </is>
       </c>
     </row>
@@ -1325,21 +1343,21 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>M3 Spacer 8mm OD 20mm Tall</t>
+          <t>M5 Spacer 8mm OD 30mm Tall</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0F8QLBKYC</t>
+          <t>https://amazon.com/dp/B0CQ53LS2B</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>6mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions. Optional: use a 6mm OD (or smaller) spacer for the one nearest each end of the Gantry X extrusion (2 total) and the stock 345mm extrusion fits without cutting.</t>
+          <t>Purchase preferred. Printed as alternative with same dimensions.</t>
         </is>
       </c>
     </row>
@@ -1350,78 +1368,78 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>M5 Spacer 8mm OD 20mm Tall</t>
+          <t>M5 Spacer 10mm OD 20mm Tall</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0CRL77N5C</t>
+          <t>https://amazon.com/dp/B0D2L3H5LV</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Purchase preferred. Printed as alternative with same dimensions.</t>
+          <t>8mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.</t>
         </is>
       </c>
     </row>
     <row r="49" s="6">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Spacers (Aluminum)</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>M5 Spacer 8mm OD 30mm Tall</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0CQ53LS2B</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>Purchase preferred. Printed as alternative with same dimensions.</t>
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Xol Toolhead Hardware</t>
         </is>
       </c>
     </row>
     <row r="50" s="6">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Spacers (Aluminum)</t>
+          <t>Xol Toolhead Hardware</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>M5 Spacer 10mm OD 20mm Tall</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0D2L3H5LV</t>
+          <t>M3 x 6mm BHCS</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>8mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.</t>
+          <t>Not required unless building the Xol carriage.</t>
         </is>
       </c>
     </row>
     <row r="51" s="6">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Xol Toolhead Hardware</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>M2 x 12mm BHCS</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Not required unless building the Xol carriage.</t>
         </is>
       </c>
     </row>
@@ -1432,11 +1450,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>M3 x 6mm BHCS</t>
+          <t>M3 x 30mm Dowel Pin</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -1446,7 +1464,7 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Not required unless building the Xol carriage.</t>
+          <t>Only dowel used by the Xol Toolhead. Not required unless building the Xol carriage.</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1479,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>M2 x 12mm BHCS</t>
+          <t>Xol 6mm Clamp</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1482,11 +1500,11 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>M3 x 30mm Dowel Pin</t>
+          <t>D2F-L Micro Switch (Endstop)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -1496,7 +1514,7 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Only dowel used by the Xol Toolhead. Not required unless building the Xol carriage.</t>
+          <t>Not required unless building the Xol carriage.</t>
         </is>
       </c>
     </row>
@@ -1507,11 +1525,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Xol 6mm Clamp</t>
+          <t>Xol-Carriage_MGN12H_MGN9H_archetype_clips</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -1526,66 +1544,48 @@
       </c>
     </row>
     <row r="56" s="6">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Xol Toolhead Hardware</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>D2F-L Micro Switch (Endstop)</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>Not required unless building the Xol carriage.</t>
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>Electronics / Endstops</t>
         </is>
       </c>
     </row>
     <row r="57" s="6">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Xol Toolhead Hardware</t>
+          <t>Electronics / Endstops</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Xol-Carriage_MGN12H_MGN9H_archetype_clips</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>D2F-L Micro Switch (Endstop)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0DBV8XGG4</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>Not required unless building the Xol carriage.</t>
+          <t>Base machine endstops (one in each back assembly).</t>
         </is>
       </c>
     </row>
     <row r="58" s="6">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>Electronics / Endstops</t>
+          <t>Linear Rails &amp; Sliders</t>
         </is>
       </c>
     </row>
     <row r="59" s="6">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Electronics / Endstops</t>
+          <t>Linear Rails &amp; Sliders</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
@@ -1593,24 +1593,34 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>D2F-L Micro Switch (Endstop)</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0DBV8XGG4</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>Base machine endstops (one in each back assembly).</t>
+          <t>MGN9H Linear Rail Slide</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Re-usable from Stock</t>
         </is>
       </c>
     </row>
     <row r="60" s="6">
-      <c r="A60" s="7" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Linear Rails &amp; Sliders</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Y MGN9H Rail 402mm</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Re-usable from Stock</t>
         </is>
       </c>
     </row>
@@ -1621,11 +1631,11 @@
         </is>
       </c>
       <c r="B61" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>MGN9H Linear Rail Slide</t>
+          <t>MGN12H Linear Rail Slide</t>
         </is>
       </c>
       <c r="D61" s="2" t="n"/>
@@ -1642,11 +1652,11 @@
         </is>
       </c>
       <c r="B62" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Y MGN9H Rail 402mm</t>
+          <t>X MGN12H Rail 406mm</t>
         </is>
       </c>
       <c r="D62" s="2" t="n"/>
@@ -1657,132 +1667,132 @@
       </c>
     </row>
     <row r="63" s="6">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Linear Rails &amp; Sliders</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>MGN12H Linear Rail Slide</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="n"/>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Re-usable from Stock</t>
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>Linear Rail Mounting Hardware</t>
         </is>
       </c>
     </row>
     <row r="64" s="6">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Linear Rails &amp; Sliders</t>
+          <t>Linear Rail Mounting Hardware</t>
         </is>
       </c>
       <c r="B64" s="3" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>X MGN12H Rail 406mm</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="n"/>
+          <t>M3 x 8mm SHCS</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0F5Q6YYWM</t>
+        </is>
+      </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Re-usable from Stock</t>
+          <t>Rail mounting screws: 10 per Y rail (20) and 8 on the X rail, one per M3 T-Nut.</t>
         </is>
       </c>
     </row>
     <row r="65" s="6">
-      <c r="A65" s="7" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>Linear Rail Mounting Hardware</t>
         </is>
       </c>
+      <c r="B65" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>M3 T-Nut</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0G2M7W3PL</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Rail mounting T-nuts: 10 per Y rail (20) and 8 on the X rail.</t>
+        </is>
+      </c>
     </row>
     <row r="66" s="6">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>Linear Rail Mounting Hardware</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>M3 x 8mm SHCS</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0F5Q6YYWM</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Rail mounting screws: 10 per Y rail (20) and 8 on the X rail, one per M3 T-Nut.</t>
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>Motors</t>
         </is>
       </c>
     </row>
     <row r="67" s="6">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Linear Rail Mounting Hardware</t>
+          <t>Motors</t>
         </is>
       </c>
       <c r="B67" s="3" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>M3 T-Nut</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0G2M7W3PL</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Rail mounting T-nuts: 10 per Y rail (20) and 8 on the X rail.</t>
-        </is>
-      </c>
+          <t>42-48 Motor 5mmx30-37mm Shaft</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
     </row>
     <row r="68" s="6">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Extrusions</t>
         </is>
       </c>
     </row>
     <row r="69" s="6">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Extrusions</t>
         </is>
       </c>
       <c r="B69" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>42-48 Motor 5mmx30-37mm Shaft</t>
+          <t>Gantry Y-Axis 2020 Extrusion 469mm</t>
         </is>
       </c>
       <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="n"/>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Stock extrusion works: the front and back motor-mount bolt holes line up with its existing holes.</t>
+        </is>
+      </c>
     </row>
     <row r="70" s="6">
-      <c r="A70" s="7" t="inlineStr">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Extrusions</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Gantry X-Axis 2020 Extrusion 342mm</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n"/>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts. The back motor-mount bolt holes line up with the stock extrusion's existing holes. To use the stock 345mm extrusion without cutting it, fit a 6mm OD (or smaller) M3 x 20mm spacer in the spot nearest each end of this extrusion (one per back corner) instead of an 8mm one. If you cut a 345mm extrusion down to 342mm, take 1.5mm off each end: the stock holes are 5mm and 23mm from each end, so an even trim keeps both ends lined up with the back motor-mount holes.</t>
         </is>
       </c>
     </row>
@@ -1793,66 +1803,66 @@
         </is>
       </c>
       <c r="B71" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Gantry Y-Axis 2020 Extrusion 469mm</t>
+          <t>Toolhead X-Axis 2020 Extrusion 426mm</t>
         </is>
       </c>
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Stock extrusion works: the front and back motor-mount bolt holes line up with its existing holes.</t>
+          <t>Stock extrusion works: the XY joint bolt holes line up with its existing holes (5mm and 25mm from each end).</t>
         </is>
       </c>
     </row>
     <row r="72" s="6">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>Extrusions</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>Gantry X-Axis 2020 Extrusion 342mm</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="n"/>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts. The back motor-mount bolt holes line up with the stock extrusion's existing holes. To use the stock 345mm extrusion without cutting it, fit a 6mm OD (or smaller) M3 x 20mm spacer in the spot nearest each end of this extrusion (one per back corner) instead of an 8mm one. If you cut a 345mm extrusion down to 342mm, take 1.5mm off each end: the stock holes are 5mm and 23mm from each end, so an even trim keeps both ends lined up with the back motor-mount holes.</t>
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>CF Plates</t>
         </is>
       </c>
     </row>
     <row r="73" s="6">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Extrusions</t>
+          <t>CF Plates</t>
         </is>
       </c>
       <c r="B73" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>XY Live Idler Spacer 5mm CF6mm</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n"/>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>Cut from the same 6mm carbon fiber plate and machined down to 5mm (no separate 5mm sheet needed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" s="6">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>CF Plates</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>Toolhead X-Axis 2020 Extrusion 426mm</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="n"/>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>Stock extrusion works: the XY joint bolt holes line up with its existing holes (5mm and 25mm from each end).</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" s="6">
-      <c r="A74" s="7" t="inlineStr">
-        <is>
-          <t>CF Plates</t>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Back Left Bottom Plate CF6mm</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n"/>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>Cut from 6mm carbon fiber</t>
         </is>
       </c>
     </row>
@@ -1863,17 +1873,17 @@
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>XY Live Idler Spacer 5mm CF6mm</t>
+          <t>Back Left Top Plate CF6mm</t>
         </is>
       </c>
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>Cut from the same 6mm carbon fiber plate and machined down to 5mm (no separate 5mm sheet needed).</t>
+          <t>Cut from 6mm carbon fiber</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1898,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Back Left Bottom Plate CF6mm</t>
+          <t>Back Right Bottom Plate CF6mm</t>
         </is>
       </c>
       <c r="D76" s="2" t="n"/>
@@ -1909,7 +1919,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Back Left Top Plate CF6mm</t>
+          <t>Back Right Top Plate CF6mm</t>
         </is>
       </c>
       <c r="D77" s="2" t="n"/>
@@ -1930,7 +1940,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Back Right Bottom Plate CF6mm</t>
+          <t>Front Left Bottom CF6mm</t>
         </is>
       </c>
       <c r="D78" s="2" t="n"/>
@@ -1951,7 +1961,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Back Right Top Plate CF6mm</t>
+          <t>Front Left Top CF6mm</t>
         </is>
       </c>
       <c r="D79" s="2" t="n"/>
@@ -1972,7 +1982,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Front Left Bottom CF6mm</t>
+          <t>Front Right Bottom CF6mm</t>
         </is>
       </c>
       <c r="D80" s="2" t="n"/>
@@ -1993,7 +2003,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Front Left Top CF6mm</t>
+          <t>Front Right Top CF6mm</t>
         </is>
       </c>
       <c r="D81" s="2" t="n"/>
@@ -2014,7 +2024,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Front Right Bottom CF6mm</t>
+          <t>XY Live Idler Left Bottom Plate CF6mm</t>
         </is>
       </c>
       <c r="D82" s="2" t="n"/>
@@ -2035,7 +2045,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Front Right Top CF6mm</t>
+          <t>XY Live Idler Left Top Plate CF6mm</t>
         </is>
       </c>
       <c r="D83" s="2" t="n"/>
@@ -2056,7 +2066,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>XY Live Idler Left Bottom Plate CF6mm</t>
+          <t>XY Live Idler Right Bottom Plate CF6mm</t>
         </is>
       </c>
       <c r="D84" s="2" t="n"/>
@@ -2077,7 +2087,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>XY Live Idler Left Top Plate CF6mm</t>
+          <t>XY Live Idler Right Top Plate CF6mm</t>
         </is>
       </c>
       <c r="D85" s="2" t="n"/>
@@ -2088,51 +2098,51 @@
       </c>
     </row>
     <row r="86" s="6">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>CF Plates</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>XY Live Idler Right Bottom Plate CF6mm</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="n"/>
-      <c r="E86" s="4" t="inlineStr">
-        <is>
-          <t>Cut from 6mm carbon fiber</t>
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>Printed Parts</t>
         </is>
       </c>
     </row>
     <row r="87" s="6">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>CF Plates</t>
+          <t>Printed Parts</t>
         </is>
       </c>
       <c r="B87" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>XY Live Idler Right Top Plate CF6mm</t>
+          <t>Tensioner Lever Arm Revised</t>
         </is>
       </c>
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>Cut from 6mm carbon fiber</t>
+          <t>Print it (Shared Components/Print Ready, holes enlarged for printing) or cut it from CF or metal (Shared Components/For Cutting, nominal size).</t>
         </is>
       </c>
     </row>
     <row r="88" s="6">
-      <c r="A88" s="7" t="inlineStr">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>Printed Parts</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Z Carriage Spacer</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="n"/>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>Check Repo</t>
         </is>
       </c>
     </row>
@@ -2143,17 +2153,17 @@
         </is>
       </c>
       <c r="B89" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Tensioner Lever Arm Revised</t>
+          <t>Back Spacer Plate 20mm</t>
         </is>
       </c>
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>Print it (Shared Components/Print Ready, holes enlarged for printing) or cut it from CF or metal (Shared Components/For Cutting, nominal size).</t>
+          <t>Check Repo</t>
         </is>
       </c>
     </row>
@@ -2164,11 +2174,11 @@
         </is>
       </c>
       <c r="B90" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Z Carriage Spacer</t>
+          <t>Front Spacer Plate 20mm</t>
         </is>
       </c>
       <c r="D90" s="2" t="n"/>
@@ -2189,7 +2199,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Back Spacer Plate 20mm</t>
+          <t>Printed Back Motor Spacer</t>
         </is>
       </c>
       <c r="D91" s="2" t="n"/>
@@ -2210,7 +2220,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Front Spacer Plate 20mm</t>
+          <t>XY Live Idler Spacer</t>
         </is>
       </c>
       <c r="D92" s="2" t="n"/>
@@ -2221,70 +2231,41 @@
       </c>
     </row>
     <row r="93" s="6">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>Printed Parts</t>
-        </is>
-      </c>
-      <c r="B93" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>Printed Back Motor Spacer</t>
-        </is>
-      </c>
+      <c r="A93" s="2" t="n"/>
+      <c r="B93" s="3" t="n"/>
+      <c r="C93" s="2" t="n"/>
       <c r="D93" s="2" t="n"/>
-      <c r="E93" s="4" t="inlineStr">
-        <is>
-          <t>Check Repo</t>
-        </is>
-      </c>
+      <c r="E93" s="4" t="n"/>
     </row>
     <row r="94" s="6">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>Printed Parts</t>
-        </is>
-      </c>
-      <c r="B94" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>XY Live Idler Spacer</t>
-        </is>
-      </c>
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="2" t="n"/>
       <c r="D94" s="2" t="n"/>
-      <c r="E94" s="4" t="inlineStr">
-        <is>
-          <t>Check Repo</t>
-        </is>
-      </c>
+      <c r="E94" s="4" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A60:E60"/>
-    <mergeCell ref="A51:E51"/>
+  <mergeCells count="20">
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A49:E49"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A36:E36"/>
-    <mergeCell ref="A88:E88"/>
-    <mergeCell ref="A70:E70"/>
-    <mergeCell ref="A65:E65"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A56:E56"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A86:E86"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A29:E29"/>
     <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A72:E72"/>
     <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A63:E63"/>
     <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A40:E40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>